<commit_message>
Fix Excel-only imports and exports and align workspace header on scroll
</commit_message>
<xml_diff>
--- a/samples/nhap-du-lieu/01_can_ho.xlsx
+++ b/samples/nhap-du-lieu/01_can_ho.xlsx
@@ -3,16 +3,72 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="24000" firstSheet="0" activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Nhap" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Huong dan" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Vi du" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Số căn hộ
+Ví dụ: A101</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Khối
+Ví dụ: A</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Tầng
+Ví dụ: 1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Diện tích (m²)
+Dùng dấu chấm cho phần thập phân.
+Ví dụ: 75.5</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Tính phí dịch vụ
+1 = có, 0 = không.
+Ví dụ: 1</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
   <si>
     <t>so_can_ho</t>
   </si>
@@ -29,7 +85,7 @@
     <t>tinh_phi_dich_vu</t>
   </si>
   <si>
-    <t>T261020X01</t>
+    <t>T261023X01</t>
   </si>
   <si>
     <t>TESTX</t>
@@ -41,7 +97,7 @@
     <t>62.50</t>
   </si>
   <si>
-    <t>T261020X02</t>
+    <t>T261023X02</t>
   </si>
   <si>
     <t>2</t>
@@ -50,7 +106,7 @@
     <t>78</t>
   </si>
   <si>
-    <t>T261020X03</t>
+    <t>T261023X03</t>
   </si>
   <si>
     <t>3</t>
@@ -68,7 +124,10 @@
     <t>Thêm căn mới và tài khoản căn hộ. Không thay đổi căn đã có. Mật khẩu mới chỉ hiện một lần sau khi lưu.</t>
   </si>
   <si>
-    <t>Điền sheet Nhap từ dòng 2. Không đổi tên cột. Các dòng ví dụ dưới đây không được nhập tự động.</t>
+    <t>MẪU TRỐNG: điền sheet Nhap từ dòng 2 trước khi tải lên. Giữ nguyên tên cột. Tối đa 100 dòng mỗi tệp.</t>
+  </si>
+  <si>
+    <t>Sheet Vi du chỉ minh họa cách điền, không được nhập tự động. Không dùng tệp xuất Chi tiết để nhập lại.</t>
   </si>
   <si>
     <t>Tên cột</t>
@@ -123,7 +182,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -135,6 +194,9 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -145,7 +207,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF14635A"/>
+        <fgColor rgb="FF171917"/>
       </patternFill>
     </fill>
   </fills>
@@ -161,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -169,6 +231,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,7 +578,7 @@
     <col min="1" max="5" width="25" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -586,120 +650,174 @@
   <autoFilter ref="A1:E4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="85" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="42" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="42" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="42" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="42" customHeight="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="4" t="s">
+    </row>
+    <row r="5" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="D5" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="D6" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>2</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" ht="36" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="B10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="D10" s="4" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="5" width="25" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>